<commit_message>
feat: add PostgreSQL JDBC extraction and pipeline verification scripts
</commit_message>
<xml_diff>
--- a/dataset_test_plan.xlsx
+++ b/dataset_test_plan.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/78607a589bfa46ec/Desktop/ALL FOLDERS/data_eng/nhs_healthcare_platform/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_17DFC6B191E6E8BF891C87C2EAB039D0583BCDA6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE181D13-AEAA-4131-83BD-3E38CA917474}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_17DFC6B191E6E8BF891C87C2EAB039D0583BCDA6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99C76D80-1528-4106-8315-181412D7EE93}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -146,6 +159,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -435,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="22.90625" bestFit="1" customWidth="1"/>
@@ -511,6 +528,12 @@
         <v>15</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B6">
+        <f>SUM(B2:B5)</f>
+        <v>105</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>